<commit_message>
feat: support width-only and height-only image placeholders
- Add @{var:width*} and @{var:*height} syntax for proportional scaling

- Split testdata into templates/ and output/ directories

- Add UTF-8 encoding config for maven-surefire-plugin

- Update test cases with dedicated template files
</commit_message>
<xml_diff>
--- a/testdata/result.xlsx
+++ b/testdata/result.xlsx
@@ -4,19 +4,20 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28125" windowHeight="12540"/>
+    <workbookView windowWidth="28800" windowHeight="12540"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="_hiddenSheet" r:id="rId7" sheetId="4" state="hidden"/>
   </sheets>
   <calcPr calcId="144525"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>标题</t>
   </si>
@@ -24,10 +25,19 @@
     <t>图片</t>
   </si>
   <si>
-    <t>标题1</t>
+    <t>枚举</t>
   </si>
   <si>
-    <t>标题2</t>
+    <t>范围</t>
+  </si>
+  <si>
+    <t>澄海区</t>
+  </si>
+  <si>
+    <t>金平区</t>
+  </si>
+  <si>
+    <t>龙湖区</t>
   </si>
 </sst>
 </file>
@@ -50,52 +60,15 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color rgb="FFFF0000"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -109,9 +82,76 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -125,9 +165,16 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
-      <sz val="13"/>
-      <color theme="3"/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -135,7 +182,7 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
+      <color rgb="FFFFFFFF"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -144,43 +191,6 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -195,25 +205,55 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799951170384838"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399945066682943"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="6" tint="0.799951170384838"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
+        <fgColor theme="8" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -231,7 +271,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399945066682943"/>
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799951170384838"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -243,85 +301,61 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399945066682943"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="7" tint="0.399945066682943"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFA5A5A5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.799951170384838"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.799951170384838"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799951170384838"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799951170384838"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
+        <fgColor theme="7" tint="0.799951170384838"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -333,49 +367,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799951170384838"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="7" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.399945066682943"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399945066682943"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -386,6 +396,15 @@
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -430,9 +449,20 @@
     <border>
       <left/>
       <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
       <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
       </bottom>
       <diagonal/>
     </border>
@@ -466,26 +496,6 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
@@ -494,145 +504,145 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="21" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="23" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="11" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -704,125 +714,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <xdr:twoCellAnchor editAs="twoCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>95250</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>1047750</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>1047750</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="Picture 1" descr="Picture"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="true"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="95250" y="95250"/>
-          <a:ext cx="952500" cy="952500"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="twoCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>95250</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>1047750</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>1047750</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1" descr="Picture"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="true"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="95250" y="95250"/>
-          <a:ext cx="952500" cy="952500"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="twoCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>1143000</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>2095500</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>1047750</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 1" descr="Picture"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="true"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip r:embed="rId3"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1143000" y="95250"/>
-          <a:ext cx="952500" cy="952500"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1112,32 +1003,40 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="1"/>
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="3"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="12.0" collapsed="false"/>
-    <col min="2" max="2" customWidth="true" width="28.75" collapsed="false"/>
+    <col min="1" max="1" customWidth="true" width="12.0"/>
+    <col min="2" max="2" customWidth="true" width="9.125"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="90.0" customHeight="true">
-      <c r="A1" t="s">
+    <row r="1" spans="1:4">
+      <c r="A1" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s" s="0">
         <v>2</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
+      <c r="D1" t="s" s="0">
+        <v>3</v>
       </c>
     </row>
-    <row r="2" ht="90.0" customHeight="true">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2"/>
-    </row>
   </sheetData>
+  <dataValidations count="2">
+    <dataValidation type="list" sqref="C2:C65536" allowBlank="true" errorStyle="stop" showErrorMessage="true" errorTitle="错误" error="枚举值错误">
+      <formula1>_hiddenSheet!$C$1:$C$3</formula1>
+    </dataValidation>
+    <dataValidation type="whole" operator="between" sqref="D2:D65536" allowBlank="true" errorStyle="stop" showErrorMessage="true" errorTitle="错误" error="范围错误">
+      <formula1>1</formula1>
+      <formula2>5</formula2>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
   <headerFooter/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1163,4 +1062,29 @@
   <pageSetup paperSize="9" orientation="portrait"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="C1:C3"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="C1" t="s" s="0">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="C2" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="C3" t="s" s="0">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
 </file>
</xml_diff>